<commit_message>
template fix and resize
</commit_message>
<xml_diff>
--- a/lib/Template.xlsx
+++ b/lib/Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10920"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Code\FNB\Change Request Template\lib\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://datasciences-my.sharepoint.com/personal/ricardo_aguiar_datasciences_co_za/Documents/Documents/Code/Change-Request-Template/lib/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE2AE605-A4D1-47DC-8296-FBE8C5FE9A64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{EE2AE605-A4D1-47DC-8296-FBE8C5FE9A64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{429948E5-BAF7-D347-A999-E77B994AE83E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -52,9 +52,6 @@
     <t>What is the complexity of the change, Risk and Impact Analysis</t>
   </si>
   <si>
-    <t xml:space="preserve">Test Plan(What needs to be tested after the completion of the Change Order(i.e. BU, Vendor, FNB Storage)). </t>
-  </si>
-  <si>
     <t>Detailed Backout Plan</t>
   </si>
   <si>
@@ -80,6 +77,9 @@
   </si>
   <si>
     <t>Has successful testing been performed for migration into Production?</t>
+  </si>
+  <si>
+    <t>Test Plan</t>
   </si>
 </sst>
 </file>
@@ -466,133 +466,139 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="108" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="106.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="106.83203125" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2"/>
     </row>
-    <row r="3" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="2"/>
     </row>
-    <row r="7" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="2"/>
     </row>
-    <row r="8" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="3"/>
     </row>
-    <row r="9" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="3"/>
     </row>
-    <row r="10" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="2"/>
     </row>
-    <row r="11" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="3"/>
-    </row>
-    <row r="12" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="3"/>
+    </row>
+    <row r="13" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="3"/>
-    </row>
-    <row r="13" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="B13" s="2"/>
+    </row>
+    <row r="14" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="2"/>
-    </row>
-    <row r="14" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="2"/>
+    </row>
+    <row r="15" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="2"/>
-    </row>
-    <row r="15" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="B15" s="2"/>
+    </row>
+    <row r="16" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="2"/>
-    </row>
-    <row r="16" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="B16" s="2"/>
+    </row>
+    <row r="17" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="2"/>
-    </row>
-    <row r="17" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="B17" s="2"/>
+    </row>
+    <row r="18" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="2"/>
-    </row>
-    <row r="18" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="B18" s="2"/>
+    </row>
+    <row r="19" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="2"/>
-    </row>
-    <row r="19" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="B19" s="3"/>
+    </row>
+    <row r="20" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="B19" s="3"/>
-    </row>
-    <row r="20" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="B20" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{b6d87b93-bf69-4fc5-885e-6e076ce4482a}" enabled="1" method="Privileged" siteId="{f8bceab8-4a5d-4fe2-b458-49f88c19fb16}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>